<commit_message>
Rename Action Gauge to Special Gauge across docs, sheets and sim
Matches the name already used in the GDD ("หลอด Special") and the Special
ability trigger, so the term is consistent everywhere.

- GDD, CLAUDE.md, simulate/README.md: Action Gauge -> Special Gauge
- Equipment/Monster/Perk sheets: same rename in descriptions and comments
  (the two "old column name" notes in the Equipment README keep the literal
  'Action Gauge' and now say (ชื่อเดิม))
- Monster sheet: Feast!H1 header Max AG -> Max SG
- sim: MaxAG -> MaxSG, maxag -> maxsg, agauge -> specgauge
  (not sgauge, which is already the Speed Gauge variable)
- sim_report.html regenerated; results identical, only timestamps differ

Left alone on purpose: the *ByActionGauge enum ids in Sumeeper_GameData.xlsx,
which need the Unity enum and the Google Sheet renamed in the same pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/game_document/Sumeeper_Equipment_Sheet.xlsx
+++ b/game_document/Sumeeper_Equipment_Sheet.xlsx
@@ -932,7 +932,7 @@
     <row r="14">
       <c r="A14" s="39" t="inlineStr">
         <is>
-          <t>2. 'Action Gauge' → 'Charge' — จำนวนช่อง Action Gauge ที่อาวุธเติมเมื่อออก action (ค่ามาก = Special เร็ว = ดี)</t>
+          <t>2. 'Action Gauge' (ชื่อเดิม) → 'Charge' — จำนวนช่อง Special Gauge ที่อาวุธเติมเมื่อออก action (ค่ามาก = Special เร็ว = ดี)</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
     <row r="19">
       <c r="A19" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Special = fire ตอน Action Gauge เต็ม</t>
+          <t xml:space="preserve">   - Special = fire ตอน Special Gauge เต็ม</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update - naming and convention again
</commit_message>
<xml_diff>
--- a/game_document/Sumeeper_Equipment_Sheet.xlsx
+++ b/game_document/Sumeeper_Equipment_Sheet.xlsx
@@ -932,7 +932,7 @@
     <row r="14">
       <c r="A14" s="39" t="inlineStr">
         <is>
-          <t>2. 'Action Gauge' (ชื่อเดิม) → 'Charge' — จำนวนช่อง Special Gauge ที่อาวุธเติมเมื่อออก action (ค่ามาก = Special เร็ว = ดี)</t>
+          <t>2. 'Action Gauge' → 'Charge' — จำนวนช่อง Action Gauge ที่อาวุธเติมเมื่อออก action (ค่ามาก = Special เร็ว = ดี)</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
     <row r="19">
       <c r="A19" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Special = fire ตอน Special Gauge เต็ม</t>
+          <t xml:space="preserve">   - Special = fire ตอน Action Gauge เต็ม</t>
         </is>
       </c>
     </row>

</xml_diff>